<commit_message>
docs(security): ajouter documentation Couche Utilisateurs et mise à jour Excel
- Docs/security/identity.md : documentation SSO Azure AD/Entra ID SAML 2.0,
  MFA (Conditional Access), Passwordless FIDO2/YubiKey, comptes de service
  et comptes locaux. Note souveraineté : alternative Keycloak on-premise.
- Docs/specs/movetodata_features.xlsx : section Sécurité (F12.1–F12.4)
  couvrant les 4 couches : Utilisateurs, API, Data, Audit.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/specs/movetodata_features.xlsx
+++ b/Docs/specs/movetodata_features.xlsx
@@ -5,54 +5,44 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonat\Documents\Bosler\Bosler_repo\Docs\specs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\movetodata\Docs\specs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A483B0C7-6312-4536-AC7C-DF07215C4D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A66343-8D70-4648-A974-2BF49120693E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="9285" windowWidth="29040" windowHeight="15720" xr2:uid="{7CDB87B6-5015-4512-B0B4-CE6386007B49}"/>
+    <workbookView xWindow="-28920" yWindow="9285" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="242">
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Catégorie</t>
+  </si>
+  <si>
+    <t>Fonctionnalité</t>
+  </si>
+  <si>
+    <t>Route</t>
+  </si>
+  <si>
+    <t>Actions testables</t>
+  </si>
+  <si>
+    <t>F1.1</t>
+  </si>
   <si>
     <t>Authentification</t>
   </si>
   <si>
-    <t>Fonctionnalité</t>
-  </si>
-  <si>
-    <t>Route</t>
-  </si>
-  <si>
-    <t>Actions testables</t>
-  </si>
-  <si>
     <t>Login local</t>
   </si>
   <si>
@@ -62,12 +52,18 @@
     <t>username/password → dashboard</t>
   </si>
   <si>
+    <t>F1.2</t>
+  </si>
+  <si>
     <t>Login SSO OAuth2</t>
   </si>
   <si>
     <t>redirect OAuth2</t>
   </si>
   <si>
+    <t>F1.3</t>
+  </si>
+  <si>
     <t>Logout</t>
   </si>
   <si>
@@ -77,6 +73,9 @@
     <t>session détruite → retour login</t>
   </si>
   <si>
+    <t>F1.4</t>
+  </si>
+  <si>
     <t>Session expirée</t>
   </si>
   <si>
@@ -86,6 +85,9 @@
     <t>message d'erreur</t>
   </si>
   <si>
+    <t>F2.1</t>
+  </si>
+  <si>
     <t>Navigation principale</t>
   </si>
   <si>
@@ -98,6 +100,9 @@
     <t>KPIs, accès rapide, activité récente</t>
   </si>
   <si>
+    <t>F2.2</t>
+  </si>
+  <si>
     <t>Favoris</t>
   </si>
   <si>
@@ -107,6 +112,9 @@
     <t>voir ressources étoilées</t>
   </si>
   <si>
+    <t>F2.3</t>
+  </si>
+  <si>
     <t>Récemment vus</t>
   </si>
   <si>
@@ -116,6 +124,9 @@
     <t>historique navigation</t>
   </si>
   <si>
+    <t>F2.4</t>
+  </si>
+  <si>
     <t>Notifications</t>
   </si>
   <si>
@@ -125,6 +136,9 @@
     <t>lire, supprimer, marquer lu (WebSocket)</t>
   </si>
   <si>
+    <t>F2.5</t>
+  </si>
+  <si>
     <t>Command Palette</t>
   </si>
   <si>
@@ -134,6 +148,9 @@
     <t>recherche rapide</t>
   </si>
   <si>
+    <t>F3.1</t>
+  </si>
+  <si>
     <t>Projets &amp; Fichiers</t>
   </si>
   <si>
@@ -146,6 +163,9 @@
     <t>lister, créer, renommer, supprimer, permissions</t>
   </si>
   <si>
+    <t>F3.2</t>
+  </si>
+  <si>
     <t>Explorateur fichiers</t>
   </si>
   <si>
@@ -155,6 +175,9 @@
     <t>tree navigation, breadcrumb, favoris</t>
   </si>
   <si>
+    <t>F3.3</t>
+  </si>
+  <si>
     <t>Éditeur code (Monaco)</t>
   </si>
   <si>
@@ -164,6 +187,9 @@
     <t>éditer, changer branche, planifier</t>
   </si>
   <si>
+    <t>F3.4</t>
+  </si>
+  <si>
     <t>DAG visuel (Bezier)</t>
   </si>
   <si>
@@ -173,6 +199,9 @@
     <t>éditeur graphique de pipeline</t>
   </si>
   <si>
+    <t>F4.1</t>
+  </si>
+  <si>
     <t>Dataset</t>
   </si>
   <si>
@@ -185,6 +214,9 @@
     <t>tableau, colonnes, statistiques</t>
   </si>
   <si>
+    <t>F4.2</t>
+  </si>
+  <si>
     <t>Build dataset</t>
   </si>
   <si>
@@ -194,12 +226,18 @@
     <t>déclencher build, voir logs</t>
   </si>
   <si>
+    <t>F4.3</t>
+  </si>
+  <si>
     <t>Upload fichier</t>
   </si>
   <si>
     <t>uploader si dataset vide</t>
   </si>
   <si>
+    <t>F4.4</t>
+  </si>
+  <si>
     <t>Schéma</t>
   </si>
   <si>
@@ -209,6 +247,9 @@
     <t>éditer et appliquer</t>
   </si>
   <si>
+    <t>F4.5</t>
+  </si>
+  <si>
     <t>Data Health</t>
   </si>
   <si>
@@ -218,6 +259,9 @@
     <t>ajouter checks, monitoring</t>
   </si>
   <si>
+    <t>F4.6</t>
+  </si>
+  <si>
     <t>Schedules dataset</t>
   </si>
   <si>
@@ -227,6 +271,9 @@
     <t>créer cron</t>
   </si>
   <si>
+    <t>F4.7</t>
+  </si>
+  <si>
     <t>Supprimer dataset</t>
   </si>
   <si>
@@ -236,6 +283,9 @@
     <t>confirmation</t>
   </si>
   <si>
+    <t>F5.1</t>
+  </si>
+  <si>
     <t>Connect (Connect Admins uniquement)</t>
   </si>
   <si>
@@ -248,6 +298,9 @@
     <t>lister, créer (PostgreSQL, MySQL, Snowflake, REST API…)</t>
   </si>
   <si>
+    <t>F5.2</t>
+  </si>
+  <si>
     <t>Source — détail</t>
   </si>
   <si>
@@ -257,6 +310,9 @@
     <t>éditer, tester connexion, parcourir données</t>
   </si>
   <si>
+    <t>F5.3</t>
+  </si>
+  <si>
     <t>Links — liste</t>
   </si>
   <si>
@@ -266,6 +322,9 @@
     <t>lister, créer (SQL query → dataset)</t>
   </si>
   <si>
+    <t>F5.4</t>
+  </si>
+  <si>
     <t>Link — détail</t>
   </si>
   <si>
@@ -275,6 +334,9 @@
     <t>éditer SQL, déclencher build</t>
   </si>
   <si>
+    <t>F5.5</t>
+  </si>
+  <si>
     <t>Agents — liste</t>
   </si>
   <si>
@@ -284,6 +346,9 @@
     <t>lister, créer</t>
   </si>
   <si>
+    <t>F5.6</t>
+  </si>
+  <si>
     <t>Agent — détail</t>
   </si>
   <si>
@@ -293,6 +358,9 @@
     <t>statut, uptime, token, sources liées</t>
   </si>
   <si>
+    <t>F6.1</t>
+  </si>
+  <si>
     <t>Visualisations Kepler</t>
   </si>
   <si>
@@ -305,6 +373,9 @@
     <t>afficher, éditer requête, sauvegarder</t>
   </si>
   <si>
+    <t>F6.2</t>
+  </si>
+  <si>
     <t>Dashboard</t>
   </si>
   <si>
@@ -314,6 +385,9 @@
     <t>multi-onglets, ajouter chart, abonnement, versioning</t>
   </si>
   <si>
+    <t>F7.1</t>
+  </si>
+  <si>
     <t>Builds &amp; Schedules</t>
   </si>
   <si>
@@ -326,6 +400,9 @@
     <t>lister, filtrer, détail logs</t>
   </si>
   <si>
+    <t>F7.2</t>
+  </si>
+  <si>
     <t>Schedules</t>
   </si>
   <si>
@@ -335,6 +412,9 @@
     <t>lister, activer/désactiver, filtrer</t>
   </si>
   <si>
+    <t>F7.3</t>
+  </si>
+  <si>
     <t>Schedule détail</t>
   </si>
   <si>
@@ -344,6 +424,9 @@
     <t>voir config cron, historique</t>
   </si>
   <si>
+    <t>F8.1</t>
+  </si>
+  <si>
     <t>Access Manager</t>
   </si>
   <si>
@@ -356,6 +439,9 @@
     <t>lister, filtrer, créer demande</t>
   </si>
   <si>
+    <t>F8.2</t>
+  </si>
+  <si>
     <t>Détail demande</t>
   </si>
   <si>
@@ -365,6 +451,9 @@
     <t>approuver / refuser</t>
   </si>
   <si>
+    <t>F9.1</t>
+  </si>
+  <si>
     <t>Paramètres utilisateur</t>
   </si>
   <si>
@@ -377,6 +466,9 @@
     <t>modifier nom, email, avatar</t>
   </si>
   <si>
+    <t>F9.2</t>
+  </si>
+  <si>
     <t>Préférences</t>
   </si>
   <si>
@@ -386,6 +478,9 @@
     <t>thème, langue, disposition</t>
   </si>
   <si>
+    <t>F9.3</t>
+  </si>
+  <si>
     <t>Tokens API</t>
   </si>
   <si>
@@ -395,6 +490,9 @@
     <t>créer, lister, révoquer</t>
   </si>
   <si>
+    <t>F9.4</t>
+  </si>
+  <si>
     <t>Changer password</t>
   </si>
   <si>
@@ -404,6 +502,9 @@
     <t>modifier (uniquement comptes locaux)</t>
   </si>
   <si>
+    <t>F9.5</t>
+  </si>
+  <si>
     <t>Groupes</t>
   </si>
   <si>
@@ -413,6 +514,9 @@
     <t>voir ses groupes</t>
   </si>
   <si>
+    <t>F9.6</t>
+  </si>
+  <si>
     <t>Activité connexion</t>
   </si>
   <si>
@@ -422,6 +526,9 @@
     <t>historique IP/device</t>
   </si>
   <si>
+    <t>F10.1</t>
+  </si>
+  <si>
     <t>Administration (platform admin)</t>
   </si>
   <si>
@@ -434,12 +541,18 @@
     <t>créer, supprimer, rôles</t>
   </si>
   <si>
+    <t>F10.2</t>
+  </si>
+  <si>
     <t>/portal/settings/groups</t>
   </si>
   <si>
     <t>créer, membres</t>
   </si>
   <si>
+    <t>F10.3</t>
+  </si>
+  <si>
     <t>SSO</t>
   </si>
   <si>
@@ -449,6 +562,9 @@
     <t>configurer SAML/OAuth2</t>
   </si>
   <si>
+    <t>F10.4</t>
+  </si>
+  <si>
     <t>Licence</t>
   </si>
   <si>
@@ -458,6 +574,9 @@
     <t>activer, copier clé</t>
   </si>
   <si>
+    <t>F10.5</t>
+  </si>
+  <si>
     <t>Thème plateforme</t>
   </si>
   <si>
@@ -467,6 +586,9 @@
     <t>logo, couleurs</t>
   </si>
   <si>
+    <t>F10.6</t>
+  </si>
+  <si>
     <t>SMTP</t>
   </si>
   <si>
@@ -476,6 +598,9 @@
     <t>configurer email</t>
   </si>
   <si>
+    <t>F10.7</t>
+  </si>
+  <si>
     <t>BackingFs</t>
   </si>
   <si>
@@ -485,6 +610,9 @@
     <t>stockage (local/S3/GCS)</t>
   </si>
   <si>
+    <t>F10.8</t>
+  </si>
+  <si>
     <t>Spark</t>
   </si>
   <si>
@@ -494,6 +622,9 @@
     <t>URL, ressources</t>
   </si>
   <si>
+    <t>F10.9</t>
+  </si>
+  <si>
     <t>Bulk users</t>
   </si>
   <si>
@@ -503,6 +634,12 @@
     <t>import CSV</t>
   </si>
   <si>
+    <t>F11.1</t>
+  </si>
+  <si>
+    <t>Features IA</t>
+  </si>
+  <si>
     <t>Text-to-SQL (F1)</t>
   </si>
   <si>
@@ -512,6 +649,9 @@
     <t>bouton IA, question → SQL généré, exécuter</t>
   </si>
   <si>
+    <t>F11.2</t>
+  </si>
+  <si>
     <t>Augmented Analytics (F2)</t>
   </si>
   <si>
@@ -521,6 +661,9 @@
     <t>sparkle → anomalies, prévision, clustering, résumé</t>
   </si>
   <si>
+    <t>F11.3</t>
+  </si>
+  <si>
     <t>Assistant conversationnel (F3)</t>
   </si>
   <si>
@@ -530,6 +673,9 @@
     <t>chat SSE, graphiques inline, historique</t>
   </si>
   <si>
+    <t>F11.4</t>
+  </si>
+  <si>
     <t>Smart Connector (F4)</t>
   </si>
   <si>
@@ -539,6 +685,9 @@
     <t>score qualité, types détectés, suggestions charts</t>
   </si>
   <si>
+    <t>F11.5</t>
+  </si>
+  <si>
     <t>Import fichiers (F5)</t>
   </si>
   <si>
@@ -548,172 +697,55 @@
     <t>drag &amp; drop, rapport, recommandations, créer dataset</t>
   </si>
   <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Catégorie</t>
-  </si>
-  <si>
-    <t>F1.1</t>
-  </si>
-  <si>
-    <t>F1.2</t>
-  </si>
-  <si>
-    <t>F1.3</t>
-  </si>
-  <si>
-    <t>F1.4</t>
-  </si>
-  <si>
-    <t>F2.1</t>
-  </si>
-  <si>
-    <t>F2.2</t>
-  </si>
-  <si>
-    <t>F2.3</t>
-  </si>
-  <si>
-    <t>F2.4</t>
-  </si>
-  <si>
-    <t>F2.5</t>
-  </si>
-  <si>
-    <t>F3.1</t>
-  </si>
-  <si>
-    <t>F3.2</t>
-  </si>
-  <si>
-    <t>F3.3</t>
-  </si>
-  <si>
-    <t>F3.4</t>
-  </si>
-  <si>
-    <t>F4.1</t>
-  </si>
-  <si>
-    <t>F4.2</t>
-  </si>
-  <si>
-    <t>F4.3</t>
-  </si>
-  <si>
-    <t>F4.4</t>
-  </si>
-  <si>
-    <t>F4.5</t>
-  </si>
-  <si>
-    <t>F4.6</t>
-  </si>
-  <si>
-    <t>F4.7</t>
-  </si>
-  <si>
-    <t>Features IA</t>
-  </si>
-  <si>
-    <t>F5.1</t>
-  </si>
-  <si>
-    <t>F5.2</t>
-  </si>
-  <si>
-    <t>F5.3</t>
-  </si>
-  <si>
-    <t>F5.4</t>
-  </si>
-  <si>
-    <t>F5.5</t>
-  </si>
-  <si>
-    <t>F5.6</t>
-  </si>
-  <si>
-    <t>F6.1</t>
-  </si>
-  <si>
-    <t>F6.2</t>
-  </si>
-  <si>
-    <t>F7.1</t>
-  </si>
-  <si>
-    <t>F7.2</t>
-  </si>
-  <si>
-    <t>F7.3</t>
-  </si>
-  <si>
-    <t>F8.1</t>
-  </si>
-  <si>
-    <t>F8.2</t>
-  </si>
-  <si>
-    <t>F9.1</t>
-  </si>
-  <si>
-    <t>F9.2</t>
-  </si>
-  <si>
-    <t>F9.3</t>
-  </si>
-  <si>
-    <t>F9.4</t>
-  </si>
-  <si>
-    <t>F9.5</t>
-  </si>
-  <si>
-    <t>F9.6</t>
-  </si>
-  <si>
-    <t>F10.1</t>
-  </si>
-  <si>
-    <t>F10.2</t>
-  </si>
-  <si>
-    <t>F10.3</t>
-  </si>
-  <si>
-    <t>F10.4</t>
-  </si>
-  <si>
-    <t>F10.5</t>
-  </si>
-  <si>
-    <t>F10.6</t>
-  </si>
-  <si>
-    <t>F10.7</t>
-  </si>
-  <si>
-    <t>F10.8</t>
-  </si>
-  <si>
-    <t>F10.9</t>
-  </si>
-  <si>
-    <t>F11.1</t>
-  </si>
-  <si>
-    <t>F11.2</t>
-  </si>
-  <si>
-    <t>F11.3</t>
-  </si>
-  <si>
-    <t>F11.4</t>
-  </si>
-  <si>
-    <t>F11.5</t>
+    <t>F12.1</t>
+  </si>
+  <si>
+    <t>Securite</t>
+  </si>
+  <si>
+    <t>Couche Utilisateurs (SSO / MFA / FIDO2)</t>
+  </si>
+  <si>
+    <t>IdP externe</t>
+  </si>
+  <si>
+    <t>SSO Azure AD/Entra ID SAML 2.0 ; MFA impose par Conditional Access ; Passwordless FIDO2/YubiKey ; voir Docs/security/identity.md</t>
+  </si>
+  <si>
+    <t>F12.2</t>
+  </si>
+  <si>
+    <t>Couche API (Rate Limiting + WAF + Security Headers)</t>
+  </si>
+  <si>
+    <t>nginx (frontend)</t>
+  </si>
+  <si>
+    <t>limit_req 30 req/min API / 10 req/min auth ; bloc SQLi/XSS via map ; headers OWASP : X-Frame-Options, CSP, X-Content-Type-Options</t>
+  </si>
+  <si>
+    <t>F12.3</t>
+  </si>
+  <si>
+    <t>Couche Data (RLS PostgreSQL + chiffrement at-rest)</t>
+  </si>
+  <si>
+    <t>boson-db (docker-compose)</t>
+  </si>
+  <si>
+    <t>POSTGRES_RLS_ENABLED=true ; ALTER TABLE ... ENABLE ROW LEVEL SECURITY cote applicatif ; chiffrement LUKS ou KMS on-premise documente dans .env.movetodata.example</t>
+  </si>
+  <si>
+    <t>F12.4</t>
+  </si>
+  <si>
+    <t>Couche Audit (logs JSON + rotation)</t>
+  </si>
+  <si>
+    <t>nginx + docker-compose</t>
+  </si>
+  <si>
+    <t>Log format JSON nginx (time, IP, method, path, status, response_time) ; log driver json-file avec max-size/max-file sur tous les services ; audit PostgreSQL (log_connections, log_statement=ddl)</t>
   </si>
 </sst>
 </file>
@@ -742,13 +774,11 @@
       <name val="Arial Unicode MS"/>
     </font>
     <font>
-      <sz val="8"/>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -759,6 +789,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE8F4F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -774,7 +809,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -784,6 +819,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1118,8 +1156,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95A756D1-D267-49C9-A916-AD5BE971770E}">
-  <dimension ref="A1:E54"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.75"/>
   <cols>
     <col min="2" max="2" width="34.953125" customWidth="1"/>
@@ -1130,924 +1168,991 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>170</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" ht="29.5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="29.5" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>171</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>172</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" ht="29.5">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="29.5" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>173</v>
+        <v>13</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>174</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="29.5">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="29.5" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>175</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>176</v>
+        <v>26</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="26">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="26" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>177</v>
+        <v>30</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="29.5">
-      <c r="A9" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="C9" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10" s="1" t="s">
-        <v>179</v>
+        <v>38</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="29.5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="29.5" customHeight="1">
       <c r="A11" s="1" t="s">
-        <v>180</v>
+        <v>42</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="29.5">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="29.5" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>181</v>
+        <v>47</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="29.5">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="29.5" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>182</v>
+        <v>51</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="29.5">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="29.5" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>183</v>
+        <v>55</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>42</v>
+        <v>57</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="29.5">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="29.5" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>184</v>
+        <v>59</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>45</v>
+        <v>61</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="29.5">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="29.5" customHeight="1">
       <c r="A16" s="1" t="s">
-        <v>185</v>
+        <v>64</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
-        <v>186</v>
+        <v>68</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>49</v>
+        <v>66</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" s="1" t="s">
-        <v>187</v>
+        <v>71</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" ht="29.5">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="29.5" customHeight="1">
       <c r="A19" s="1" t="s">
-        <v>188</v>
+        <v>75</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>56</v>
+        <v>76</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>57</v>
+        <v>77</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>58</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" s="1" t="s">
-        <v>189</v>
+        <v>79</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>59</v>
+        <v>80</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>61</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
-        <v>190</v>
+        <v>83</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>62</v>
+        <v>84</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>63</v>
+        <v>85</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="44.25">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="44.25" customHeight="1">
       <c r="A22" s="1" t="s">
-        <v>192</v>
+        <v>87</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" ht="29.5">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="29.5" customHeight="1">
       <c r="A23" s="1" t="s">
-        <v>193</v>
+        <v>92</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" ht="29.5">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="29.5" customHeight="1">
       <c r="A24" s="1" t="s">
-        <v>194</v>
+        <v>96</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>72</v>
+        <v>97</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="29.5">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="29.5" customHeight="1">
       <c r="A25" s="1" t="s">
-        <v>195</v>
+        <v>100</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>75</v>
+        <v>101</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" ht="26">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="26" customHeight="1">
       <c r="A26" s="1" t="s">
-        <v>196</v>
+        <v>104</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="29.5">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="29.5" customHeight="1">
       <c r="A27" s="1" t="s">
-        <v>197</v>
+        <v>108</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>81</v>
+        <v>109</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="29.5">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="29.5" customHeight="1">
       <c r="A28" s="1" t="s">
-        <v>198</v>
+        <v>112</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>85</v>
+        <v>114</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>86</v>
+        <v>115</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" ht="44.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" ht="44.25" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>199</v>
+        <v>117</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>89</v>
+        <v>119</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>90</v>
+        <v>120</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A31" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A32" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A33" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="26" customHeight="1">
+      <c r="A34" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A35" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A36" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" ht="26" customHeight="1">
+      <c r="A37" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A38" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" ht="26" customHeight="1">
+      <c r="A39" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" ht="26" customHeight="1">
+      <c r="A40" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="26" customHeight="1">
+      <c r="A41" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="26" customHeight="1">
+      <c r="A42" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" ht="26" customHeight="1">
+      <c r="A43" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" ht="26" customHeight="1">
+      <c r="A44" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" ht="26" customHeight="1">
+      <c r="A45" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" ht="26" customHeight="1">
+      <c r="A46" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="26" customHeight="1">
+      <c r="A47" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="26" customHeight="1">
+      <c r="A48" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" ht="39" customHeight="1">
+      <c r="A49" s="1" t="s">
         <v>200</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E30" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" ht="29.5">
-      <c r="A31" s="1" t="s">
+      <c r="B49" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="C49" s="1" t="s">
         <v>201</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C31" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" ht="29.5">
-      <c r="A32" s="1" t="s">
+      <c r="D49" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="E32" s="1" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="29.5">
-      <c r="A33" s="1" t="s">
+      <c r="E49" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="26">
-      <c r="A34" s="1" t="s">
+    </row>
+    <row r="50" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A50" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" ht="29.5">
-      <c r="A35" s="1" t="s">
+      <c r="B50" t="s">
         <v>205</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" ht="29.5">
-      <c r="A36" s="1" t="s">
+      <c r="C50" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" ht="26">
-      <c r="A37" s="1" t="s">
+      <c r="D50" s="1" t="s">
         <v>207</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" ht="29.5">
-      <c r="A38" s="1" t="s">
+      <c r="E50" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>119</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" ht="26">
-      <c r="A39" s="1" t="s">
+    </row>
+    <row r="51" spans="1:5" ht="44.25" customHeight="1">
+      <c r="A51" s="1" t="s">
         <v>209</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" ht="26">
-      <c r="A40" s="1" t="s">
+      <c r="B51" t="s">
+        <v>205</v>
+      </c>
+      <c r="C51" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>125</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="26">
-      <c r="A41" s="1" t="s">
+      <c r="D51" s="1" t="s">
         <v>211</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="26">
-      <c r="A42" s="1" t="s">
+      <c r="E51" s="1" t="s">
         <v>212</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" ht="26">
-      <c r="A43" s="1" t="s">
+    </row>
+    <row r="52" spans="1:5" ht="29.5" customHeight="1">
+      <c r="A52" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>134</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" ht="26">
-      <c r="A44" s="1" t="s">
+      <c r="B52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C52" s="1" t="s">
         <v>214</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" ht="26">
-      <c r="A45" s="1" t="s">
+      <c r="D52" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B45" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" ht="26">
-      <c r="A46" s="1" t="s">
+      <c r="E52" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="B46" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="D46" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" ht="26">
-      <c r="A47" s="1" t="s">
+    </row>
+    <row r="53" spans="1:5" ht="44.25" customHeight="1">
+      <c r="A53" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="B47" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>146</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" ht="26">
-      <c r="A48" s="1" t="s">
+      <c r="B53" t="s">
+        <v>205</v>
+      </c>
+      <c r="C53" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="B48" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="D48" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="E48" s="1" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" ht="39">
-      <c r="A49" s="1" t="s">
+      <c r="D53" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B49" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="D49" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="E49" s="1" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" ht="29.5">
-      <c r="A50" s="1" t="s">
+      <c r="E53" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B50" t="s">
-        <v>191</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="D50" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="E50" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" ht="44.25">
-      <c r="A51" s="1" t="s">
+    </row>
+    <row r="54" spans="1:5" ht="44.25" customHeight="1">
+      <c r="A54" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="B51" t="s">
-        <v>191</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="D51" s="1" t="s">
-        <v>158</v>
-      </c>
-      <c r="E51" s="1" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" ht="29.5">
-      <c r="A52" s="1" t="s">
+      <c r="B54" t="s">
+        <v>205</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B52" t="s">
-        <v>191</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="D52" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="E52" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" ht="44.25">
-      <c r="A53" s="1" t="s">
+      <c r="D54" s="1" t="s">
         <v>223</v>
       </c>
-      <c r="B53" t="s">
-        <v>191</v>
-      </c>
-      <c r="C53" s="1" t="s">
-        <v>163</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" ht="44.25">
-      <c r="A54" s="1" t="s">
+      <c r="E54" s="1" t="s">
         <v>224</v>
       </c>
-      <c r="B54" t="s">
-        <v>191</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>168</v>
+    </row>
+    <row r="55" spans="1:5" ht="103.25">
+      <c r="A55" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" ht="88.5">
+      <c r="A56" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" ht="132.75">
+      <c r="A57" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="132.75">
+      <c r="A58" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>241</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>